<commit_message>
fixed the missing jx:area header
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/competitionResults/_FlatFile.xlsx
+++ b/owlcms/src/main/resources/templates/competitionResults/_FlatFile.xlsx
@@ -76,6 +76,19 @@
     <author>Jean-François Lamy</author>
   </authors>
   <commentList>
+    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{DA3EAA0E-9611-469E-9C9E-A573FD5AC14C}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>jx:area(lastCell="V10")</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="A2" authorId="0" shapeId="0" xr:uid="{F0A7DC28-4FBA-4A0F-B1F3-C337DC82D113}">
       <text>
         <r>
@@ -85,8 +98,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>jx:each(items="athletes" var="group" groupBy="group.categorySortCode" groupOrder="ASC" lastCell="W2")
-jx:each(items="group.items" var="l"  varIndex="lifterLoop" lastCell="W2")</t>
+          <t>jx:each(items="athletes" var="l" lastCell="V2")</t>
         </r>
       </text>
     </comment>

</xml_diff>